<commit_message>
Replace project reference sheet with 18-09-26 0002
</commit_message>
<xml_diff>
--- a/reference/demo.xlsx
+++ b/reference/demo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="36">
   <si>
     <t xml:space="preserve">Customer Signature                                                                                                                          Authorized Signature </t>
   </si>
@@ -85,6 +85,9 @@
     <t>Mob: 01718-306103, 01724-358341</t>
   </si>
   <si>
+    <t>18.09.2026</t>
+  </si>
+  <si>
     <t>Officer BNC AGRO CARE Area Manager</t>
   </si>
   <si>
@@ -95,6 +98,30 @@
   </si>
   <si>
     <t>Reg. Office kajolgouri, khorna,Shajahanpur,bogura</t>
+  </si>
+  <si>
+    <t>NC-Darma</t>
+  </si>
+  <si>
+    <t>100 ml x 30 bot.</t>
+  </si>
+  <si>
+    <t>M/s Master Traders</t>
+  </si>
+  <si>
+    <t>Nem: Alz.Aktaruzzaman (nannu)</t>
+  </si>
+  <si>
+    <t>Add: Subotbazar,Kolakopa, Gabtoli,Bogura</t>
+  </si>
+  <si>
+    <t>Mobile: 01947-615107</t>
+  </si>
+  <si>
+    <t>NC-Vit</t>
+  </si>
+  <si>
+    <t>100ml x 30 bot</t>
   </si>
 </sst>
 </file>
@@ -691,120 +718,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -856,6 +769,120 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1188,70 +1215,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" s="15" customFormat="1" ht="45" x14ac:dyDescent="0.3">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="75" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="79"/>
-      <c r="C1" s="79"/>
-      <c r="D1" s="79"/>
-      <c r="E1" s="79"/>
-      <c r="F1" s="79"/>
-      <c r="G1" s="79"/>
-      <c r="H1" s="79"/>
-      <c r="I1" s="79"/>
-      <c r="J1" s="79"/>
-      <c r="K1" s="79"/>
-      <c r="L1" s="80"/>
+      <c r="B1" s="76"/>
+      <c r="C1" s="76"/>
+      <c r="D1" s="76"/>
+      <c r="E1" s="76"/>
+      <c r="F1" s="76"/>
+      <c r="G1" s="76"/>
+      <c r="H1" s="76"/>
+      <c r="I1" s="76"/>
+      <c r="J1" s="76"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="77"/>
     </row>
     <row r="2" spans="1:16" s="15" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="81" t="s">
-        <v>26</v>
-      </c>
-      <c r="B2" s="82"/>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
-      <c r="I2" s="82"/>
-      <c r="J2" s="82"/>
-      <c r="K2" s="82"/>
-      <c r="L2" s="83"/>
+      <c r="A2" s="78" t="s">
+        <v>27</v>
+      </c>
+      <c r="B2" s="79"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
+      <c r="F2" s="79"/>
+      <c r="G2" s="79"/>
+      <c r="H2" s="79"/>
+      <c r="I2" s="79"/>
+      <c r="J2" s="79"/>
+      <c r="K2" s="79"/>
+      <c r="L2" s="80"/>
     </row>
     <row r="3" spans="1:16" s="15" customFormat="1" ht="14.45" x14ac:dyDescent="0.3">
-      <c r="A3" s="84" t="s">
+      <c r="A3" s="81" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="85"/>
-      <c r="C3" s="85"/>
-      <c r="D3" s="85"/>
-      <c r="E3" s="85"/>
-      <c r="F3" s="85"/>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="85"/>
-      <c r="J3" s="85"/>
-      <c r="K3" s="85"/>
-      <c r="L3" s="86"/>
+      <c r="B3" s="82"/>
+      <c r="C3" s="82"/>
+      <c r="D3" s="82"/>
+      <c r="E3" s="82"/>
+      <c r="F3" s="82"/>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="82"/>
+      <c r="J3" s="82"/>
+      <c r="K3" s="82"/>
+      <c r="L3" s="83"/>
     </row>
     <row r="4" spans="1:16" s="15" customFormat="1" ht="18.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="27" t="s">
         <v>16</v>
       </c>
-      <c r="B4" s="87" t="s">
+      <c r="B4" s="84" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="87"/>
-      <c r="D4" s="87"/>
-      <c r="E4" s="87"/>
-      <c r="F4" s="87"/>
-      <c r="G4" s="87"/>
-      <c r="H4" s="87"/>
-      <c r="I4" s="87"/>
-      <c r="J4" s="87"/>
-      <c r="K4" s="87"/>
-      <c r="L4" s="88"/>
+      <c r="C4" s="84"/>
+      <c r="D4" s="84"/>
+      <c r="E4" s="84"/>
+      <c r="F4" s="84"/>
+      <c r="G4" s="84"/>
+      <c r="H4" s="84"/>
+      <c r="I4" s="84"/>
+      <c r="J4" s="84"/>
+      <c r="K4" s="84"/>
+      <c r="L4" s="85"/>
     </row>
     <row r="5" spans="1:16" ht="24.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5" s="26" t="s">
@@ -1260,94 +1287,104 @@
       <c r="B5" s="25">
         <v>2</v>
       </c>
-      <c r="C5" s="89" t="s">
+      <c r="C5" s="86" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="90"/>
-      <c r="E5" s="90"/>
-      <c r="F5" s="90"/>
-      <c r="G5" s="90"/>
-      <c r="H5" s="91"/>
+      <c r="D5" s="87"/>
+      <c r="E5" s="87"/>
+      <c r="F5" s="87"/>
+      <c r="G5" s="87"/>
+      <c r="H5" s="88"/>
       <c r="I5" s="24" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="92"/>
-      <c r="K5" s="93"/>
-      <c r="L5" s="94"/>
+      <c r="J5" s="89" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="90"/>
+      <c r="L5" s="91"/>
     </row>
     <row r="6" spans="1:16" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A6" s="66"/>
-      <c r="B6" s="66"/>
-      <c r="C6" s="66"/>
-      <c r="D6" s="66"/>
-      <c r="E6" s="66"/>
-      <c r="F6" s="66"/>
-      <c r="G6" s="66"/>
-      <c r="H6" s="67"/>
-      <c r="I6" s="70" t="s">
-        <v>25</v>
-      </c>
-      <c r="J6" s="71"/>
-      <c r="K6" s="71"/>
-      <c r="L6" s="72"/>
+      <c r="A6" s="101" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="101"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="102"/>
+      <c r="I6" s="105" t="s">
+        <v>26</v>
+      </c>
+      <c r="J6" s="106"/>
+      <c r="K6" s="106"/>
+      <c r="L6" s="107"/>
       <c r="M6" s="40"/>
       <c r="N6" s="40"/>
       <c r="O6" s="40"/>
       <c r="P6" s="40"/>
     </row>
     <row r="7" spans="1:16" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A7" s="68"/>
-      <c r="B7" s="68"/>
-      <c r="C7" s="68"/>
-      <c r="D7" s="68"/>
-      <c r="E7" s="68"/>
-      <c r="F7" s="68"/>
-      <c r="G7" s="68"/>
-      <c r="H7" s="69"/>
-      <c r="I7" s="70" t="s">
-        <v>23</v>
-      </c>
-      <c r="J7" s="71"/>
-      <c r="K7" s="71"/>
-      <c r="L7" s="72"/>
+      <c r="A7" s="103" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="103"/>
+      <c r="C7" s="103"/>
+      <c r="D7" s="103"/>
+      <c r="E7" s="103"/>
+      <c r="F7" s="103"/>
+      <c r="G7" s="103"/>
+      <c r="H7" s="104"/>
+      <c r="I7" s="105" t="s">
+        <v>24</v>
+      </c>
+      <c r="J7" s="106"/>
+      <c r="K7" s="106"/>
+      <c r="L7" s="107"/>
       <c r="M7" s="40"/>
       <c r="N7" s="40"/>
       <c r="O7" s="40"/>
       <c r="P7" s="40"/>
     </row>
     <row r="8" spans="1:16" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A8" s="69"/>
-      <c r="B8" s="73"/>
-      <c r="C8" s="73"/>
-      <c r="D8" s="73"/>
-      <c r="E8" s="73"/>
-      <c r="F8" s="73"/>
-      <c r="G8" s="73"/>
-      <c r="H8" s="74"/>
-      <c r="I8" s="63" t="s">
-        <v>24</v>
-      </c>
-      <c r="J8" s="64"/>
-      <c r="K8" s="64"/>
-      <c r="L8" s="65"/>
+      <c r="A8" s="104" t="s">
+        <v>32</v>
+      </c>
+      <c r="B8" s="108"/>
+      <c r="C8" s="108"/>
+      <c r="D8" s="108"/>
+      <c r="E8" s="108"/>
+      <c r="F8" s="108"/>
+      <c r="G8" s="108"/>
+      <c r="H8" s="109"/>
+      <c r="I8" s="98" t="s">
+        <v>25</v>
+      </c>
+      <c r="J8" s="99"/>
+      <c r="K8" s="99"/>
+      <c r="L8" s="100"/>
       <c r="M8" s="41"/>
       <c r="N8" s="41"/>
       <c r="O8" s="41"/>
       <c r="P8" s="41"/>
     </row>
     <row r="9" spans="1:16" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="61"/>
-      <c r="B9" s="61"/>
-      <c r="C9" s="61"/>
-      <c r="D9" s="61"/>
-      <c r="E9" s="61"/>
-      <c r="F9" s="61"/>
-      <c r="G9" s="61"/>
-      <c r="H9" s="62"/>
-      <c r="I9" s="75"/>
-      <c r="J9" s="76"/>
-      <c r="K9" s="76"/>
-      <c r="L9" s="77"/>
+      <c r="A9" s="96" t="s">
+        <v>33</v>
+      </c>
+      <c r="B9" s="96"/>
+      <c r="C9" s="96"/>
+      <c r="D9" s="96"/>
+      <c r="E9" s="96"/>
+      <c r="F9" s="96"/>
+      <c r="G9" s="96"/>
+      <c r="H9" s="97"/>
+      <c r="I9" s="110"/>
+      <c r="J9" s="111"/>
+      <c r="K9" s="111"/>
+      <c r="L9" s="112"/>
       <c r="M9" s="42"/>
     </row>
     <row r="10" spans="1:16" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1399,11 +1436,21 @@
       <c r="A11" s="54">
         <v>1</v>
       </c>
-      <c r="B11" s="55"/>
-      <c r="C11" s="50"/>
-      <c r="D11" s="36"/>
-      <c r="E11" s="34"/>
-      <c r="F11" s="35"/>
+      <c r="B11" s="55" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="50" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" s="36">
+        <v>1</v>
+      </c>
+      <c r="E11" s="34">
+        <v>56</v>
+      </c>
+      <c r="F11" s="35">
+        <v>560</v>
+      </c>
       <c r="G11" s="30"/>
       <c r="H11" s="44"/>
       <c r="I11" s="33"/>
@@ -1418,11 +1465,21 @@
       <c r="A12" s="43">
         <v>2</v>
       </c>
-      <c r="B12" s="49"/>
-      <c r="C12" s="50"/>
-      <c r="D12" s="36"/>
-      <c r="E12" s="34"/>
-      <c r="F12" s="35"/>
+      <c r="B12" s="49" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="50" t="s">
+        <v>29</v>
+      </c>
+      <c r="D12" s="36">
+        <v>1</v>
+      </c>
+      <c r="E12" s="34">
+        <v>56</v>
+      </c>
+      <c r="F12" s="35">
+        <v>560</v>
+      </c>
       <c r="G12" s="30"/>
       <c r="H12" s="24"/>
       <c r="I12" s="33"/>
@@ -1453,10 +1510,10 @@
       <c r="O13" s="23"/>
     </row>
     <row r="14" spans="1:16" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="59">
+      <c r="A14" s="94">
         <v>4</v>
       </c>
-      <c r="B14" s="57"/>
+      <c r="B14" s="92"/>
       <c r="C14" s="50"/>
       <c r="D14" s="36"/>
       <c r="E14" s="34"/>
@@ -1472,8 +1529,8 @@
       <c r="O14" s="23"/>
     </row>
     <row r="15" spans="1:16" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="60"/>
-      <c r="B15" s="58"/>
+      <c r="A15" s="95"/>
+      <c r="B15" s="93"/>
       <c r="C15" s="50"/>
       <c r="D15" s="36"/>
       <c r="E15" s="34"/>
@@ -1490,24 +1547,24 @@
     </row>
     <row r="16" spans="1:16" s="15" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A16" s="20"/>
-      <c r="B16" s="96" t="s">
+      <c r="B16" s="58" t="s">
         <v>6</v>
       </c>
-      <c r="C16" s="97"/>
+      <c r="C16" s="59"/>
       <c r="D16" s="43">
         <f>SUM(D11:D15)</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E16" s="20"/>
       <c r="F16" s="31">
         <f>SUM(F11:F15)</f>
-        <v>0</v>
+        <v>1120</v>
       </c>
       <c r="G16" s="22"/>
-      <c r="H16" s="98" t="s">
+      <c r="H16" s="60" t="s">
         <v>6</v>
       </c>
-      <c r="I16" s="99"/>
+      <c r="I16" s="61"/>
       <c r="J16" s="29"/>
       <c r="K16" s="20"/>
       <c r="L16" s="32">
@@ -1526,26 +1583,26 @@
     </row>
     <row r="17" spans="1:15" s="15" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A17" s="20"/>
-      <c r="B17" s="100" t="s">
+      <c r="B17" s="62" t="s">
         <v>5</v>
       </c>
-      <c r="C17" s="101"/>
+      <c r="C17" s="63"/>
       <c r="D17" s="37">
         <f>D16+J16</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E17" s="21"/>
       <c r="F17" s="31"/>
       <c r="G17" s="28"/>
       <c r="H17" s="28"/>
-      <c r="I17" s="102" t="s">
+      <c r="I17" s="64" t="s">
         <v>4</v>
       </c>
-      <c r="J17" s="102"/>
-      <c r="K17" s="102"/>
+      <c r="J17" s="64"/>
+      <c r="K17" s="64"/>
       <c r="L17" s="48">
         <f>F16+L16</f>
-        <v>0</v>
+        <v>1120</v>
       </c>
       <c r="M17" s="16"/>
       <c r="N17" s="15" t="e">
@@ -1559,55 +1616,55 @@
     </row>
     <row r="18" spans="1:15" s="15" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="20"/>
-      <c r="B18" s="103" t="s">
+      <c r="B18" s="65" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="104"/>
-      <c r="D18" s="104"/>
-      <c r="E18" s="104"/>
-      <c r="F18" s="104"/>
-      <c r="G18" s="104"/>
-      <c r="H18" s="104"/>
-      <c r="I18" s="104"/>
-      <c r="J18" s="104"/>
-      <c r="K18" s="104"/>
+      <c r="C18" s="66"/>
+      <c r="D18" s="66"/>
+      <c r="E18" s="66"/>
+      <c r="F18" s="66"/>
+      <c r="G18" s="66"/>
+      <c r="H18" s="66"/>
+      <c r="I18" s="66"/>
+      <c r="J18" s="66"/>
+      <c r="K18" s="66"/>
       <c r="L18" s="38"/>
       <c r="M18" s="16"/>
     </row>
     <row r="19" spans="1:15" s="15" customFormat="1" ht="19.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="20"/>
-      <c r="B19" s="105" t="s">
+      <c r="B19" s="67" t="s">
         <v>3</v>
       </c>
-      <c r="C19" s="102"/>
-      <c r="D19" s="102"/>
-      <c r="E19" s="102"/>
-      <c r="F19" s="102"/>
-      <c r="G19" s="102"/>
-      <c r="H19" s="102"/>
-      <c r="I19" s="102"/>
-      <c r="J19" s="102"/>
-      <c r="K19" s="102"/>
+      <c r="C19" s="64"/>
+      <c r="D19" s="64"/>
+      <c r="E19" s="64"/>
+      <c r="F19" s="64"/>
+      <c r="G19" s="64"/>
+      <c r="H19" s="64"/>
+      <c r="I19" s="64"/>
+      <c r="J19" s="64"/>
+      <c r="K19" s="64"/>
       <c r="L19" s="39">
         <f>L17-L18</f>
-        <v>0</v>
+        <v>1120</v>
       </c>
       <c r="M19" s="16"/>
     </row>
     <row r="20" spans="1:15" s="15" customFormat="1" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A20" s="19"/>
-      <c r="B20" s="106" t="s">
+      <c r="B20" s="68" t="s">
         <v>2</v>
       </c>
-      <c r="C20" s="106"/>
-      <c r="D20" s="107"/>
-      <c r="E20" s="108"/>
-      <c r="F20" s="108"/>
-      <c r="G20" s="108"/>
-      <c r="H20" s="108"/>
-      <c r="I20" s="108"/>
-      <c r="J20" s="108"/>
-      <c r="K20" s="109"/>
+      <c r="C20" s="68"/>
+      <c r="D20" s="69"/>
+      <c r="E20" s="70"/>
+      <c r="F20" s="70"/>
+      <c r="G20" s="70"/>
+      <c r="H20" s="70"/>
+      <c r="I20" s="70"/>
+      <c r="J20" s="70"/>
+      <c r="K20" s="71"/>
       <c r="L20" s="28"/>
       <c r="M20" s="16"/>
       <c r="N20" s="15" t="e">
@@ -1683,11 +1740,11 @@
     <row r="24" spans="1:15" s="15" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="17"/>
       <c r="B24" s="6"/>
-      <c r="C24" s="112" t="s">
+      <c r="C24" s="74" t="s">
         <v>19</v>
       </c>
-      <c r="D24" s="112"/>
-      <c r="E24" s="112"/>
+      <c r="D24" s="74"/>
+      <c r="E24" s="74"/>
       <c r="F24" s="1"/>
       <c r="G24" s="17"/>
       <c r="H24" s="17"/>
@@ -1721,52 +1778,52 @@
       <c r="M25" s="7"/>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="A26" s="110" t="s">
+      <c r="A26" s="72" t="s">
         <v>1</v>
       </c>
-      <c r="B26" s="110"/>
-      <c r="C26" s="110"/>
-      <c r="D26" s="110"/>
-      <c r="E26" s="110"/>
-      <c r="F26" s="110"/>
-      <c r="G26" s="110"/>
-      <c r="H26" s="110"/>
-      <c r="I26" s="110"/>
-      <c r="J26" s="110"/>
-      <c r="K26" s="110"/>
-      <c r="L26" s="110"/>
+      <c r="B26" s="72"/>
+      <c r="C26" s="72"/>
+      <c r="D26" s="72"/>
+      <c r="E26" s="72"/>
+      <c r="F26" s="72"/>
+      <c r="G26" s="72"/>
+      <c r="H26" s="72"/>
+      <c r="I26" s="72"/>
+      <c r="J26" s="72"/>
+      <c r="K26" s="72"/>
+      <c r="L26" s="72"/>
       <c r="M26" s="7"/>
     </row>
     <row r="27" spans="1:15" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="111" t="s">
+      <c r="A27" s="73" t="s">
         <v>0</v>
       </c>
-      <c r="B27" s="111"/>
-      <c r="C27" s="111"/>
-      <c r="D27" s="111"/>
-      <c r="E27" s="111"/>
-      <c r="F27" s="111"/>
-      <c r="G27" s="111"/>
-      <c r="H27" s="111"/>
-      <c r="I27" s="111"/>
-      <c r="J27" s="111"/>
-      <c r="K27" s="111"/>
-      <c r="L27" s="111"/>
+      <c r="B27" s="73"/>
+      <c r="C27" s="73"/>
+      <c r="D27" s="73"/>
+      <c r="E27" s="73"/>
+      <c r="F27" s="73"/>
+      <c r="G27" s="73"/>
+      <c r="H27" s="73"/>
+      <c r="I27" s="73"/>
+      <c r="J27" s="73"/>
+      <c r="K27" s="73"/>
+      <c r="L27" s="73"/>
       <c r="M27" s="7"/>
     </row>
     <row r="28" spans="1:15" ht="18" x14ac:dyDescent="0.25">
-      <c r="A28" s="95"/>
-      <c r="B28" s="95"/>
-      <c r="C28" s="95"/>
-      <c r="D28" s="95"/>
-      <c r="E28" s="95"/>
-      <c r="F28" s="95"/>
-      <c r="G28" s="95"/>
-      <c r="H28" s="95"/>
-      <c r="I28" s="95"/>
-      <c r="J28" s="95"/>
-      <c r="K28" s="95"/>
-      <c r="L28" s="95"/>
+      <c r="A28" s="57"/>
+      <c r="B28" s="57"/>
+      <c r="C28" s="57"/>
+      <c r="D28" s="57"/>
+      <c r="E28" s="57"/>
+      <c r="F28" s="57"/>
+      <c r="G28" s="57"/>
+      <c r="H28" s="57"/>
+      <c r="I28" s="57"/>
+      <c r="J28" s="57"/>
+      <c r="K28" s="57"/>
+      <c r="L28" s="57"/>
       <c r="M28" s="7"/>
     </row>
     <row r="29" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
@@ -1827,6 +1884,22 @@
     </row>
   </sheetData>
   <mergeCells count="28">
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="A14:A15"/>
+    <mergeCell ref="A9:H9"/>
+    <mergeCell ref="I8:L8"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="I6:L6"/>
+    <mergeCell ref="I7:L7"/>
+    <mergeCell ref="A8:H8"/>
+    <mergeCell ref="I9:L9"/>
+    <mergeCell ref="A1:L1"/>
+    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A3:L3"/>
+    <mergeCell ref="B4:L4"/>
+    <mergeCell ref="C5:H5"/>
+    <mergeCell ref="J5:L5"/>
     <mergeCell ref="A28:L28"/>
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="H16:I16"/>
@@ -1839,22 +1912,6 @@
     <mergeCell ref="A26:L26"/>
     <mergeCell ref="A27:L27"/>
     <mergeCell ref="C24:E24"/>
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
-    <mergeCell ref="A3:L3"/>
-    <mergeCell ref="B4:L4"/>
-    <mergeCell ref="C5:H5"/>
-    <mergeCell ref="J5:L5"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="A14:A15"/>
-    <mergeCell ref="A9:H9"/>
-    <mergeCell ref="I8:L8"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="I6:L6"/>
-    <mergeCell ref="I7:L7"/>
-    <mergeCell ref="A8:H8"/>
-    <mergeCell ref="I9:L9"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A3" r:id="rId1" display="mailto:bengalcropcare@gmail.com"/>

</xml_diff>